<commit_message>
Add DIvehi Field and calender field support
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dev2026\mosh-forms-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BC0D5D-F94A-435D-8508-D6A5FF621D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3F4FEE-0FD8-49D4-A04F-313263C09681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2805" yWindow="2805" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>Name</t>
   </si>
@@ -43,6 +43,18 @@
   </si>
   <si>
     <t>Name2</t>
+  </si>
+  <si>
+    <t>Dhivehi Name</t>
+  </si>
+  <si>
+    <t>{divehi.name}</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>{date.startdate}</t>
   </si>
 </sst>
 </file>
@@ -428,10 +440,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D5:F6"/>
+  <dimension ref="D5:H6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="5" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
         <v>4</v>
       </c>
@@ -441,8 +456,14 @@
       <c r="F5" t="s">
         <v>1</v>
       </c>
+      <c r="G5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>2</v>
       </c>
@@ -451,6 +472,12 @@
       </c>
       <c r="F6" t="s">
         <v>3</v>
+      </c>
+      <c r="G6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct current and next date
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dev2026\mosh-forms-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3F4FEE-0FD8-49D4-A04F-313263C09681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C05EF19-2152-4C02-A8A1-984299CDFBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2805" yWindow="2805" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>Name</t>
   </si>
@@ -55,19 +55,55 @@
   </si>
   <si>
     <t>{date.startdate}</t>
+  </si>
+  <si>
+    <t>{date_current_10}</t>
+  </si>
+  <si>
+    <t>{date_divehi_current_10}</t>
+  </si>
+  <si>
+    <t>date_divehi_current_10</t>
+  </si>
+  <si>
+    <t>date_current_10</t>
+  </si>
+  <si>
+    <t>{date_next_5}</t>
+  </si>
+  <si>
+    <t>date_next_5</t>
+  </si>
+  <si>
+    <t>{date_divehi_next_5}</t>
+  </si>
+  <si>
+    <t>date_divehi_next_5</t>
+  </si>
+  <si>
+    <t>{some_date_field}</t>
+  </si>
+  <si>
+    <t>some_date_field</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFF9FAFB"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -90,8 +126,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,13 +477,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D5:H6"/>
+  <dimension ref="D5:M6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
         <v>4</v>
       </c>
@@ -462,8 +504,23 @@
       <c r="H5" t="s">
         <v>7</v>
       </c>
+      <c r="I5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J5" t="s">
+        <v>11</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="6" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>2</v>
       </c>
@@ -478,9 +535,25 @@
       </c>
       <c r="H6" t="s">
         <v>8</v>
+      </c>
+      <c r="I6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed RTL(Dhivehi SUpport) for Date FIelds
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dev2026\mosh-forms-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C05EF19-2152-4C02-A8A1-984299CDFBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0BD748-9E0D-47C8-8563-43093B5665BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2805" yWindow="2805" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>Name</t>
   </si>
@@ -85,6 +85,12 @@
   </si>
   <si>
     <t>some_date_field</t>
+  </si>
+  <si>
+    <t>Diveh Date</t>
+  </si>
+  <si>
+    <t>{date}</t>
   </si>
 </sst>
 </file>
@@ -477,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D5:M6"/>
+  <dimension ref="B5:M6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -488,7 +494,10 @@
     <col min="12" max="12" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="4:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
       <c r="D5" t="s">
         <v>4</v>
       </c>
@@ -520,7 +529,10 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="4:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
       <c r="D6" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Added date range selection
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dev2026\mosh-forms-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0BD748-9E0D-47C8-8563-43093B5665BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966FCBB2-C831-4AA9-AA92-C21B572669AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2805" yWindow="2805" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Name</t>
   </si>
@@ -91,6 +91,45 @@
   </si>
   <si>
     <t>{date}</t>
+  </si>
+  <si>
+    <t>Date Range</t>
+  </si>
+  <si>
+    <t>{date_many_1}</t>
+  </si>
+  <si>
+    <t>{date_many_2}</t>
+  </si>
+  <si>
+    <t>{date_many_3}</t>
+  </si>
+  <si>
+    <t>{date_many_4}</t>
+  </si>
+  <si>
+    <t>{date_many_5}</t>
+  </si>
+  <si>
+    <t>{date_many_6}</t>
+  </si>
+  <si>
+    <t>{date_many_7}</t>
+  </si>
+  <si>
+    <t>{date_many_8}</t>
+  </si>
+  <si>
+    <t>{date_many_9}</t>
+  </si>
+  <si>
+    <t>{date_many_10}</t>
+  </si>
+  <si>
+    <t>{date_many_11}</t>
+  </si>
+  <si>
+    <t>{date_many_12}</t>
   </si>
 </sst>
 </file>
@@ -483,85 +522,147 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B5:M6"/>
+  <dimension ref="B5:O17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
         <v>19</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>4</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>0</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>1</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>5</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>7</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" t="s">
         <v>12</v>
       </c>
-      <c r="J5" t="s">
+      <c r="L5" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>2</v>
       </c>
-      <c r="E6" t="s">
+      <c r="G6" t="s">
         <v>2</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>3</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>6</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>8</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>9</v>
       </c>
-      <c r="J6" t="s">
+      <c r="L6" t="s">
         <v>10</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="N6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>